<commit_message>
vault backup: 2026-03-31 21:33:36
</commit_message>
<xml_diff>
--- a/附件/2026年发展党员需求统计表 1.xlsx
+++ b/附件/2026年发展党员需求统计表 1.xlsx
@@ -2002,7 +2002,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" ht="60" spans="1:18">
+    <row r="7" ht="21" customHeight="1" spans="1:18">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" ht="60" spans="1:18">
+    <row r="8" ht="19" customHeight="1" spans="1:18">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" ht="30" spans="1:18">
+    <row r="10" ht="15" spans="1:18">
       <c r="A10" s="3">
         <v>8</v>
       </c>

</xml_diff>